<commit_message>
Large update for bug and functionallities
</commit_message>
<xml_diff>
--- a/assets/TEMPLATE.xlsx
+++ b/assets/TEMPLATE.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.guinamard\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.guinamard\Documents\GitHub\MWQuote\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB384AF4-C02C-4B7D-BE06-7A90B86D01E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C130731C-40D3-4A20-80C6-2041BD809072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1230" yWindow="2670" windowWidth="21600" windowHeight="11295" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OFFRE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$M$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$M$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
   <si>
     <t xml:space="preserve">Devis N° / Quote ref : </t>
   </si>
@@ -113,7 +113,19 @@
     <t>PU_REF</t>
   </si>
   <si>
-    <t>COMMENT_REF</t>
+    <t>TOOL_REF</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>PTOOL_REF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMMENT_REF </t>
+  </si>
+  <si>
+    <t>CUSTOMER_NAME</t>
   </si>
 </sst>
 </file>
@@ -493,26 +505,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -523,6 +530,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -538,14 +551,13 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -910,7 +922,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:P44"/>
+  <dimension ref="A2:P45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
@@ -930,19 +942,19 @@
       <c r="H2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="50" t="s">
+      <c r="K2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="51"/>
+      <c r="L2" s="48"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="57" t="s">
+      <c r="K3" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="51"/>
+      <c r="L3" s="48"/>
     </row>
     <row r="4" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M4" s="6"/>
@@ -953,17 +965,17 @@
       <c r="B6" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="44"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="43"/>
       <c r="H6" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="44"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="43"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
@@ -976,7 +988,9 @@
         <v>4</v>
       </c>
       <c r="F8" s="7"/>
-      <c r="H8" s="3"/>
+      <c r="H8" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="L8" s="7"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -1019,50 +1033,50 @@
         <v>5</v>
       </c>
       <c r="D14" s="11"/>
-      <c r="E14" s="54" t="s">
+      <c r="E14" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="43"/>
+      <c r="F14" s="41"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
       <c r="L14" s="12" t="s">
         <v>8</v>
       </c>
       <c r="M14" s="9"/>
     </row>
     <row r="15" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="55"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="45">
+      <c r="B15" s="54"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="60">
         <v>1000</v>
       </c>
-      <c r="F15" s="46"/>
+      <c r="F15" s="45"/>
       <c r="G15" s="24"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="48" t="s">
+      <c r="I15" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="J15" s="46"/>
+      <c r="J15" s="45"/>
       <c r="K15" s="5"/>
       <c r="L15" s="8"/>
     </row>
     <row r="17" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="41"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="59"/>
       <c r="I17" s="14" t="s">
         <v>10</v>
       </c>
@@ -1081,14 +1095,14 @@
       <c r="B18" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="53" t="s">
+      <c r="C18" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="43"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1121,7 +1135,7 @@
       <c r="J21" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K21" s="58" t="s">
+      <c r="K21" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L21" s="2" t="e">
@@ -1140,7 +1154,7 @@
       <c r="J22" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K22" s="58" t="s">
+      <c r="K22" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L22" s="2" t="e">
@@ -1159,7 +1173,7 @@
       <c r="J23" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L23" s="2" t="e">
@@ -1178,7 +1192,7 @@
       <c r="J24" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K24" s="58" t="s">
+      <c r="K24" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L24" s="2" t="e">
@@ -1197,7 +1211,7 @@
       <c r="J25" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K25" s="58" t="s">
+      <c r="K25" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L25" s="2" t="e">
@@ -1216,7 +1230,7 @@
       <c r="J26" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K26" s="58" t="s">
+      <c r="K26" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L26" s="2" t="e">
@@ -1235,7 +1249,7 @@
       <c r="J27" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K27" s="58" t="s">
+      <c r="K27" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L27" s="2" t="e">
@@ -1254,7 +1268,7 @@
       <c r="J28" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K28" s="58" t="s">
+      <c r="K28" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L28" s="2" t="e">
@@ -1273,7 +1287,7 @@
       <c r="J29" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="58" t="s">
+      <c r="K29" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L29" s="2" t="e">
@@ -1292,7 +1306,7 @@
       <c r="J30" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K30" s="58" t="s">
+      <c r="K30" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L30" s="2" t="e">
@@ -1379,119 +1393,138 @@
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B37" s="36"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="25"/>
-      <c r="J37" s="25"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="27"/>
-    </row>
-    <row r="38" spans="2:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="56"/>
-      <c r="C38" s="43"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="43"/>
-      <c r="I38" s="43"/>
-      <c r="J38" s="43"/>
-      <c r="K38" s="43"/>
-      <c r="L38" s="43"/>
-    </row>
-    <row r="39" spans="2:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="52" t="s">
+      <c r="B37" s="3"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="18"/>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B38" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="K38" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="L38" s="27" t="str">
+        <f>K38</f>
+        <v>PTOOL_REF</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="55"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
+      <c r="H39" s="41"/>
+      <c r="I39" s="41"/>
+      <c r="J39" s="41"/>
+      <c r="K39" s="41"/>
+      <c r="L39" s="41"/>
+    </row>
+    <row r="40" spans="2:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C39" s="51"/>
-      <c r="D39" s="51"/>
-      <c r="E39" s="51"/>
-      <c r="F39" s="51"/>
-      <c r="G39" s="51"/>
-      <c r="H39" s="51"/>
-      <c r="I39" s="51"/>
-      <c r="J39" s="51"/>
-      <c r="K39" s="51"/>
-      <c r="L39" s="51"/>
-    </row>
-    <row r="40" spans="2:12" ht="291" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="60"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="60"/>
-      <c r="L40" s="60"/>
-    </row>
-    <row r="41" spans="2:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
-      <c r="H41" s="29"/>
-      <c r="I41" s="30"/>
-      <c r="J41" s="30"/>
-      <c r="K41" s="31"/>
-      <c r="L41" s="31"/>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="19"/>
-      <c r="J42" s="19"/>
-      <c r="K42" s="21"/>
-      <c r="L42" s="21"/>
-    </row>
-    <row r="44" spans="2:12" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="47" t="s">
+      <c r="C40" s="48"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="48"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="48"/>
+      <c r="H40" s="48"/>
+      <c r="I40" s="48"/>
+      <c r="J40" s="48"/>
+      <c r="K40" s="48"/>
+      <c r="L40" s="48"/>
+    </row>
+    <row r="41" spans="2:12" ht="291" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" s="51"/>
+      <c r="D41" s="51"/>
+      <c r="E41" s="51"/>
+      <c r="F41" s="51"/>
+      <c r="G41" s="51"/>
+      <c r="H41" s="51"/>
+      <c r="I41" s="51"/>
+      <c r="J41" s="51"/>
+      <c r="K41" s="51"/>
+      <c r="L41" s="51"/>
+    </row>
+    <row r="42" spans="2:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="30"/>
+      <c r="J42" s="30"/>
+      <c r="K42" s="31"/>
+      <c r="L42" s="31"/>
+    </row>
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
+      <c r="K43" s="21"/>
+      <c r="L43" s="21"/>
+    </row>
+    <row r="45" spans="2:12" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="C44" s="43"/>
-      <c r="D44" s="43"/>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="43"/>
-      <c r="I44" s="43"/>
-      <c r="J44" s="43"/>
-      <c r="K44" s="43"/>
-      <c r="L44" s="43"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="41"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="41"/>
+      <c r="J45" s="41"/>
+      <c r="K45" s="41"/>
+      <c r="L45" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B45:L45"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I14:K14"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B39:L39"/>
     <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="C18:H18"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B39:L39"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B44:L44"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I14:K14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125978" footer="0.31496062992125978"/>

</xml_diff>

<commit_message>
Enhance project management features: add database backup and restore functionality, improve project display names, and update .gitignore. Remove unused clipboard image save script.
</commit_message>
<xml_diff>
--- a/assets/TEMPLATE.xlsx
+++ b/assets/TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.guinamard\Documents\GitHub\MWQuote\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C130731C-40D3-4A20-80C6-2041BD809072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81768489-FA0F-45E6-B2E8-430659529BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="OFFRE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$M$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$N$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="30">
   <si>
     <t xml:space="preserve">Devis N° / Quote ref : </t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>CUSTOMER_NAME</t>
+  </si>
+  <si>
+    <t>IMAGE_PREVIEW</t>
   </si>
 </sst>
 </file>
@@ -413,7 +416,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
@@ -481,15 +484,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -502,11 +496,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -515,27 +531,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -555,7 +562,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -922,7 +928,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:P45"/>
+  <dimension ref="A2:Q46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
@@ -930,60 +936,64 @@
     <col min="5" max="5" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="2.7109375" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="10" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" customWidth="1"/>
-    <col min="13" max="13" width="3.140625" customWidth="1"/>
-    <col min="15" max="15" width="16.140625" customWidth="1"/>
+    <col min="9" max="9" width="1.85546875" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" customWidth="1"/>
+    <col min="11" max="11" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.85546875" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
+    <col min="14" max="14" width="3.140625" customWidth="1"/>
+    <col min="16" max="16" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H2" s="35" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="47" t="s">
+      <c r="I2" s="32"/>
+      <c r="L2" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="48"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H3" s="35" t="s">
+      <c r="M2" s="53"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="56" t="s">
+      <c r="I3" s="32"/>
+      <c r="L3" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="48"/>
-    </row>
-    <row r="4" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="M4" s="6"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="32"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="42" t="s">
+      <c r="M3" s="53"/>
+    </row>
+    <row r="4" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N4" s="6"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="29"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B6" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="43"/>
-      <c r="H6" s="42" t="s">
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="49"/>
+      <c r="H6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="43"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I6" s="48"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="49"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="F7" s="7"/>
       <c r="H7" s="3"/>
-      <c r="L7" s="7"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M7" s="7"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
@@ -991,27 +1001,28 @@
       <c r="H8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="L8" s="7"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M8" s="7"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" s="22"/>
       <c r="F9" s="7"/>
       <c r="H9" s="22"/>
-      <c r="L9" s="7"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I9" s="39"/>
+      <c r="M9" s="7"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B10" s="3"/>
       <c r="F10" s="7"/>
       <c r="H10" s="3"/>
-      <c r="L10" s="7"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M10" s="7"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B11" s="3"/>
       <c r="F11" s="7"/>
       <c r="H11" s="3"/>
-      <c r="L11" s="7"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M11" s="7"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -1021,514 +1032,536 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="L12" s="8"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="O13" s="32"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="L12" s="5"/>
+      <c r="M12" s="8"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="P13" s="29"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="B14" s="10"/>
       <c r="C14" s="23" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="11"/>
-      <c r="E14" s="53" t="s">
+      <c r="E14" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="41"/>
+      <c r="F14" s="46"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
-      <c r="I14" s="46" t="s">
+      <c r="I14" s="11"/>
+      <c r="J14" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="12" t="s">
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="M14" s="9"/>
-    </row>
-    <row r="15" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="54"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="60">
+      <c r="N14" s="9"/>
+    </row>
+    <row r="15" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="56"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="61">
         <v>1000</v>
       </c>
-      <c r="F15" s="45"/>
+      <c r="F15" s="51"/>
       <c r="G15" s="24"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="44" t="s">
+      <c r="I15" s="5"/>
+      <c r="J15" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="J15" s="45"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="8"/>
-    </row>
-    <row r="17" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K15" s="51"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="8"/>
+    </row>
+    <row r="17" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="58"/>
-      <c r="F17" s="58"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="14" t="s">
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="36"/>
+      <c r="J17" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J17" s="14" t="s">
+      <c r="K17" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K17" s="15" t="s">
+      <c r="L17" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="M17" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="M17" s="13"/>
-    </row>
-    <row r="18" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="34" t="s">
+      <c r="N17" s="13"/>
+    </row>
+    <row r="18" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="52" t="s">
+      <c r="C18" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="1"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="7"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
-      <c r="L18" s="7"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L18" s="1"/>
+      <c r="M18" s="7"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="17"/>
+      <c r="I19" s="7"/>
       <c r="J19" s="17"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="18"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K19" s="17"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="18"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="2"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="17"/>
       <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="28" t="s">
+      <c r="I21" s="7"/>
+      <c r="J21" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="K21" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K21" s="39" t="s">
+      <c r="L21" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L21" s="2" t="e">
-        <f t="shared" ref="L21:L25" si="0">K21*I21</f>
+      <c r="M21" s="2" t="e">
+        <f t="shared" ref="M21:M25" si="0">L21*J21</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H22" s="7"/>
-      <c r="I22" s="28" t="s">
+      <c r="I22" s="7"/>
+      <c r="J22" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J22" s="17" t="s">
+      <c r="K22" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K22" s="39" t="s">
+      <c r="L22" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L22" s="2" t="e">
+      <c r="M22" s="2" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="28" t="s">
+      <c r="I23" s="7"/>
+      <c r="J23" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J23" s="17" t="s">
+      <c r="K23" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K23" s="39" t="s">
+      <c r="L23" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L23" s="2" t="e">
+      <c r="M23" s="2" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="7"/>
-      <c r="I24" s="28" t="s">
+      <c r="I24" s="7"/>
+      <c r="J24" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J24" s="17" t="s">
+      <c r="K24" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K24" s="39" t="s">
+      <c r="L24" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L24" s="2" t="e">
+      <c r="M24" s="2" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H25" s="7"/>
-      <c r="I25" s="28" t="s">
+      <c r="I25" s="7"/>
+      <c r="J25" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J25" s="17" t="s">
+      <c r="K25" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K25" s="39" t="s">
+      <c r="L25" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L25" s="2" t="e">
+      <c r="M25" s="2" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H26" s="7"/>
-      <c r="I26" s="28" t="s">
+      <c r="I26" s="7"/>
+      <c r="J26" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J26" s="17" t="s">
+      <c r="K26" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K26" s="39" t="s">
+      <c r="L26" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L26" s="2" t="e">
-        <f t="shared" ref="L26" si="1">K26*I26</f>
+      <c r="M26" s="2" t="e">
+        <f t="shared" ref="M26" si="1">L26*J26</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H27" s="7"/>
-      <c r="I27" s="28" t="s">
+      <c r="I27" s="7"/>
+      <c r="J27" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J27" s="17" t="s">
+      <c r="K27" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K27" s="39" t="s">
+      <c r="L27" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L27" s="2" t="e">
-        <f t="shared" ref="L27:L28" si="2">K27*I27</f>
+      <c r="M27" s="2" t="e">
+        <f t="shared" ref="M27:M28" si="2">L27*J27</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H28" s="7"/>
-      <c r="I28" s="28" t="s">
+      <c r="I28" s="7"/>
+      <c r="J28" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J28" s="17" t="s">
+      <c r="K28" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K28" s="39" t="s">
+      <c r="L28" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L28" s="2" t="e">
+      <c r="M28" s="2" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H29" s="7"/>
-      <c r="I29" s="28" t="s">
+      <c r="I29" s="7"/>
+      <c r="J29" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J29" s="17" t="s">
+      <c r="K29" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="39" t="s">
+      <c r="L29" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L29" s="2" t="e">
-        <f t="shared" ref="L29" si="3">K29*I29</f>
+      <c r="M29" s="2" t="e">
+        <f t="shared" ref="M29" si="3">L29*J29</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H30" s="7"/>
-      <c r="I30" s="28" t="s">
+      <c r="I30" s="7"/>
+      <c r="J30" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J30" s="17" t="s">
+      <c r="K30" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K30" s="39" t="s">
+      <c r="L30" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="L30" s="2" t="e">
-        <f t="shared" ref="L30:L36" si="4">K30*I30</f>
+      <c r="M30" s="2" t="e">
+        <f t="shared" ref="M30:M36" si="4">L30*J30</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="17" t="s">
+      <c r="I31" s="7"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2">
+      <c r="L31" s="2"/>
+      <c r="M31" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="17" t="s">
+      <c r="I32" s="7"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2">
+      <c r="L32" s="2"/>
+      <c r="M32" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="3"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="17" t="s">
+      <c r="I33" s="7"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2">
+      <c r="L33" s="2"/>
+      <c r="M33" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="3"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="17" t="s">
+      <c r="I34" s="7"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2">
+      <c r="L34" s="2"/>
+      <c r="M34" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="3"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="17" t="s">
+      <c r="I35" s="7"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2">
+      <c r="L35" s="2"/>
+      <c r="M35" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="3"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="28"/>
-      <c r="J36" s="17" t="s">
+      <c r="I36" s="7"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2">
+      <c r="L36" s="2"/>
+      <c r="M36" s="2">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" s="3"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="17"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="18"/>
-    </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="36" t="s">
+      <c r="I37" s="7"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="18"/>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B38" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="28" t="s">
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="40"/>
+      <c r="J38" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="J38" s="25" t="s">
+      <c r="K38" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="K38" s="26" t="s">
+      <c r="L38" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="L38" s="27" t="str">
-        <f>K38</f>
+      <c r="M38" s="27" t="str">
+        <f>L38</f>
         <v>PTOOL_REF</v>
       </c>
     </row>
-    <row r="39" spans="2:12" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="55"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
-      <c r="H39" s="41"/>
-      <c r="I39" s="41"/>
-      <c r="J39" s="41"/>
-      <c r="K39" s="41"/>
-      <c r="L39" s="41"/>
-    </row>
-    <row r="40" spans="2:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="49" t="s">
+    <row r="39" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="57"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="46"/>
+      <c r="H39" s="46"/>
+      <c r="I39" s="46"/>
+      <c r="J39" s="46"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="46"/>
+      <c r="M39" s="46"/>
+    </row>
+    <row r="40" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
-      <c r="J40" s="48"/>
-      <c r="K40" s="48"/>
-      <c r="L40" s="48"/>
-    </row>
-    <row r="41" spans="2:12" ht="291" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="50" t="s">
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="44"/>
+      <c r="I40" s="38"/>
+    </row>
+    <row r="41" spans="2:13" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="C41" s="51"/>
-      <c r="D41" s="51"/>
-      <c r="E41" s="51"/>
-      <c r="F41" s="51"/>
-      <c r="G41" s="51"/>
-      <c r="H41" s="51"/>
-      <c r="I41" s="51"/>
-      <c r="J41" s="51"/>
-      <c r="K41" s="51"/>
-      <c r="L41" s="51"/>
-    </row>
-    <row r="42" spans="2:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="30"/>
-      <c r="J42" s="30"/>
-      <c r="K42" s="31"/>
-      <c r="L42" s="31"/>
-    </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="19"/>
-      <c r="J43" s="19"/>
-      <c r="K43" s="21"/>
-      <c r="L43" s="21"/>
-    </row>
-    <row r="45" spans="2:12" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="40" t="s">
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="42"/>
+      <c r="I41" s="37"/>
+      <c r="J41" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+    </row>
+    <row r="42" spans="2:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="41"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="41"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="42"/>
+      <c r="I42" s="37"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="13"/>
+    </row>
+    <row r="43" spans="2:13" ht="170.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="41"/>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="42"/>
+      <c r="I43" s="37"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="13"/>
+      <c r="L43" s="13"/>
+      <c r="M43" s="13"/>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="19"/>
+      <c r="K44" s="19"/>
+      <c r="L44" s="21"/>
+      <c r="M44" s="21"/>
+    </row>
+    <row r="46" spans="2:13" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="C45" s="41"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="41"/>
-      <c r="F45" s="41"/>
-      <c r="G45" s="41"/>
-      <c r="H45" s="41"/>
-      <c r="I45" s="41"/>
-      <c r="J45" s="41"/>
-      <c r="K45" s="41"/>
-      <c r="L45" s="41"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="46"/>
+      <c r="E46" s="46"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="46"/>
+      <c r="H46" s="46"/>
+      <c r="I46" s="46"/>
+      <c r="J46" s="46"/>
+      <c r="K46" s="46"/>
+      <c r="L46" s="46"/>
+      <c r="M46" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B45:L45"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B40:L40"/>
-    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="L2:M2"/>
     <mergeCell ref="C18:H18"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B39:L39"/>
-    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="B39:M39"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B41:H43"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B46:M46"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J14:L14"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125978" footer="0.31496062992125978"/>
-  <pageSetup paperSize="9" scale="75" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
export multiple tool cost
</commit_message>
<xml_diff>
--- a/assets/TEMPLATE.xlsx
+++ b/assets/TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.guinamard\Documents\GitHub\MWQuote\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CFEA4D-0689-4940-A9C9-9536FD64503E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C67E77-C6F4-4B87-916D-E30F2E499431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="OFFRE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$N$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFRE!$A$1:$N$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="30">
   <si>
     <t xml:space="preserve">Devis N° / Quote ref : </t>
   </si>
@@ -414,7 +414,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
@@ -510,65 +510,86 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -933,7 +954,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:Q46"/>
+  <dimension ref="A2:Q49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
@@ -955,20 +976,20 @@
         <v>0</v>
       </c>
       <c r="I2" s="32"/>
-      <c r="L2" s="40" t="s">
+      <c r="L2" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="41"/>
+      <c r="M2" s="57"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H3" s="32" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="32"/>
-      <c r="L3" s="48" t="s">
+      <c r="L3" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="M3" s="41"/>
+      <c r="M3" s="57"/>
     </row>
     <row r="4" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="N4" s="6"/>
@@ -976,21 +997,21 @@
       <c r="Q4" s="29"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="50"/>
-      <c r="H6" s="49" t="s">
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="48"/>
+      <c r="H6" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="57"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="50"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
+      <c r="M6" s="48"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
@@ -1050,53 +1071,53 @@
         <v>5</v>
       </c>
       <c r="D14" s="11"/>
-      <c r="E14" s="44" t="s">
+      <c r="E14" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="43"/>
+      <c r="F14" s="45"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
-      <c r="J14" s="57" t="s">
+      <c r="J14" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
+      <c r="K14" s="45"/>
+      <c r="L14" s="45"/>
       <c r="M14" s="12" t="s">
         <v>8</v>
       </c>
       <c r="N14" s="9"/>
     </row>
     <row r="15" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="45"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="51">
+      <c r="B15" s="59"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="62">
         <v>1000</v>
       </c>
-      <c r="F15" s="46"/>
+      <c r="F15" s="50"/>
       <c r="G15" s="24"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="58" t="s">
+      <c r="J15" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="K15" s="46"/>
+      <c r="K15" s="50"/>
       <c r="L15" s="5"/>
       <c r="M15" s="8"/>
     </row>
     <row r="17" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
-      <c r="B17" s="60" t="s">
+      <c r="B17" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="62"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="55"/>
       <c r="J17" s="14" t="s">
         <v>10</v>
       </c>
@@ -1115,15 +1136,15 @@
       <c r="B18" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="C18" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="59"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="59"/>
-      <c r="H18" s="59"/>
-      <c r="I18" s="42"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="52"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
@@ -1422,147 +1443,222 @@
       <c r="M37" s="18"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B38" s="33" t="s">
+      <c r="B38" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34"/>
-      <c r="H38" s="34"/>
+      <c r="C38" s="63"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="63"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="63"/>
       <c r="I38" s="39"/>
       <c r="J38" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K38" s="25" t="s">
+      <c r="K38" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="L38" s="26" t="s">
+      <c r="L38" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="M38" s="27" t="str">
+      <c r="M38" s="67" t="str">
         <f>L38</f>
         <v>PTOOL_REF</v>
       </c>
     </row>
-    <row r="39" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="47"/>
-      <c r="C39" s="43"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="43"/>
-      <c r="I39" s="43"/>
-      <c r="J39" s="43"/>
-      <c r="K39" s="43"/>
-      <c r="L39" s="43"/>
-      <c r="M39" s="43"/>
-    </row>
-    <row r="40" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54" t="s">
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B39" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
+      <c r="E39" s="63"/>
+      <c r="F39" s="63"/>
+      <c r="G39" s="63"/>
+      <c r="H39" s="63"/>
+      <c r="I39" s="39"/>
+      <c r="J39" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K39" s="65" t="s">
+        <v>25</v>
+      </c>
+      <c r="L39" s="66" t="s">
+        <v>26</v>
+      </c>
+      <c r="M39" s="67" t="str">
+        <f>L39</f>
+        <v>PTOOL_REF</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B40" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="63"/>
+      <c r="F40" s="63"/>
+      <c r="G40" s="63"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="39"/>
+      <c r="J40" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K40" s="65" t="s">
+        <v>25</v>
+      </c>
+      <c r="L40" s="66" t="s">
+        <v>26</v>
+      </c>
+      <c r="M40" s="67" t="str">
+        <f>L40</f>
+        <v>PTOOL_REF</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B41" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+      <c r="E41" s="34"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="34"/>
+      <c r="H41" s="34"/>
+      <c r="I41" s="68"/>
+      <c r="J41" s="69" t="s">
+        <v>22</v>
+      </c>
+      <c r="K41" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="L41" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="M41" s="27" t="str">
+        <f>L41</f>
+        <v>PTOOL_REF</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="60"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="45"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="45"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="45"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+    </row>
+    <row r="43" spans="2:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
-      <c r="G40" s="54"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="37"/>
-    </row>
-    <row r="41" spans="2:13" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="52" t="s">
+      <c r="C43" s="42"/>
+      <c r="D43" s="42"/>
+      <c r="E43" s="42"/>
+      <c r="F43" s="42"/>
+      <c r="G43" s="42"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="37"/>
+    </row>
+    <row r="44" spans="2:13" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="52"/>
-      <c r="H41" s="53"/>
-      <c r="I41" s="36"/>
-      <c r="J41" s="13" t="s">
+      <c r="C44" s="40"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="36"/>
+      <c r="J44" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="K41" s="13"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="13"/>
-    </row>
-    <row r="42" spans="2:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="52"/>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="52"/>
-      <c r="G42" s="52"/>
-      <c r="H42" s="53"/>
-      <c r="I42" s="36"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="13"/>
-    </row>
-    <row r="43" spans="2:13" ht="170.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="52"/>
-      <c r="C43" s="52"/>
-      <c r="D43" s="52"/>
-      <c r="E43" s="52"/>
-      <c r="F43" s="52"/>
-      <c r="G43" s="52"/>
-      <c r="H43" s="53"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="13"/>
-    </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="19"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="21"/>
-      <c r="M44" s="21"/>
-    </row>
-    <row r="46" spans="2:13" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="56" t="s">
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="13"/>
+    </row>
+    <row r="45" spans="2:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="36"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="13"/>
+    </row>
+    <row r="46" spans="2:13" ht="170.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="40"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="40"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="36"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
+      <c r="I47" s="20"/>
+      <c r="J47" s="19"/>
+      <c r="K47" s="19"/>
+      <c r="L47" s="21"/>
+      <c r="M47" s="21"/>
+    </row>
+    <row r="49" spans="2:13" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="43"/>
-      <c r="I46" s="43"/>
-      <c r="J46" s="43"/>
-      <c r="K46" s="43"/>
-      <c r="L46" s="43"/>
-      <c r="M46" s="43"/>
+      <c r="C49" s="45"/>
+      <c r="D49" s="45"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="45"/>
+      <c r="G49" s="45"/>
+      <c r="H49" s="45"/>
+      <c r="I49" s="45"/>
+      <c r="J49" s="45"/>
+      <c r="K49" s="45"/>
+      <c r="L49" s="45"/>
+      <c r="M49" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B41:H43"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B46:M46"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B42:M42"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B44:H46"/>
+    <mergeCell ref="B43:H43"/>
+    <mergeCell ref="B49:M49"/>
     <mergeCell ref="H6:M6"/>
     <mergeCell ref="J15:K15"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="C18:I18"/>
     <mergeCell ref="B17:I17"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B39:M39"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="E15:F15"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125978" footer="0.31496062992125978"/>

</xml_diff>